<commit_message>
Basis of Design and Process Design Report (md + pdf), tighter product splits
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/00-basis/CFU-000-PR-HMB-001_Heat-Material-Balance.xlsx
+++ b/deliverables/00-basis/CFU-000-PR-HMB-001_Heat-Material-Balance.xlsx
@@ -1418,25 +1418,25 @@
         <v>30</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>136.1</v>
+        <v>136.4</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>121.1</v>
+        <v>121.4</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>106.1</v>
+        <v>106.4</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>136.1</v>
+        <v>136.4</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>273.5</v>
+        <v>274</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>365.6</v>
+        <v>365.7</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>134.8</v>
+        <v>133.8</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>45</v>
@@ -1451,13 +1451,13 @@
         <v>45</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>153.3</v>
+        <v>152.8</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>238.5</v>
+        <v>240</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>312.6</v>
+        <v>313.9</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>45</v>
@@ -1469,13 +1469,13 @@
         <v>60</v>
       </c>
       <c r="T8" s="5" t="n">
-        <v>348.6</v>
+        <v>348.7</v>
       </c>
       <c r="U8" s="5" t="n">
         <v>350</v>
       </c>
       <c r="V8" s="5" t="n">
-        <v>398.3</v>
+        <v>398.4</v>
       </c>
       <c r="W8" s="5" t="n">
         <v>70</v>
@@ -1654,64 +1654,64 @@
         <v>569197</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>228876</v>
+        <v>229224</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>101108</v>
+        <v>101310</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>114757</v>
+        <v>114910</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>13011</v>
+        <v>13004</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>166946</v>
+        <v>166764</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>209213</v>
+        <v>208349</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>166306</v>
+        <v>165727</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>68744</v>
+        <v>68595</v>
       </c>
       <c r="R10" s="5" t="n">
-        <v>81587</v>
+        <v>81613</v>
       </c>
       <c r="S10" s="5" t="n">
-        <v>45715</v>
+        <v>45847</v>
       </c>
       <c r="T10" s="5" t="n">
-        <v>257071</v>
+        <v>256909</v>
       </c>
       <c r="U10" s="5" t="n">
-        <v>11687</v>
+        <v>11681</v>
       </c>
       <c r="V10" s="5" t="n">
-        <v>258218</v>
+        <v>258055</v>
       </c>
       <c r="W10" s="5" t="n">
-        <v>3021</v>
+        <v>3020</v>
       </c>
       <c r="X10" s="5" t="n">
-        <v>50683</v>
+        <v>50356</v>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>90231</v>
+        <v>90396</v>
       </c>
       <c r="Z10" s="5" t="n">
-        <v>7901</v>
+        <v>7894</v>
       </c>
       <c r="AA10" s="5" t="n">
-        <v>108256</v>
+        <v>108263</v>
       </c>
       <c r="AB10" s="5" t="n">
-        <v>12145</v>
+        <v>12141</v>
       </c>
       <c r="AC10" s="5" t="n">
         <v>102</v>
@@ -1723,16 +1723,16 @@
         <v>6468</v>
       </c>
       <c r="AF10" s="5" t="n">
-        <v>108290</v>
+        <v>108442</v>
       </c>
       <c r="AG10" s="5" t="n">
         <v>27607</v>
       </c>
       <c r="AH10" s="5" t="n">
-        <v>80682</v>
+        <v>80835</v>
       </c>
       <c r="AI10" s="5" t="n">
-        <v>6459</v>
+        <v>6443</v>
       </c>
     </row>
     <row r="11">
@@ -1763,61 +1763,61 @@
         <v>567874</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>215865</v>
+        <v>216219</v>
       </c>
       <c r="J11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>101108</v>
+        <v>101310</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>114757</v>
+        <v>114910</v>
       </c>
       <c r="M11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>166946</v>
+        <v>166764</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>209213</v>
+        <v>208349</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>166306</v>
+        <v>165727</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>68744</v>
+        <v>68595</v>
       </c>
       <c r="R11" s="5" t="n">
-        <v>81587</v>
+        <v>81613</v>
       </c>
       <c r="S11" s="5" t="n">
-        <v>45715</v>
+        <v>45847</v>
       </c>
       <c r="T11" s="5" t="n">
-        <v>257071</v>
+        <v>256909</v>
       </c>
       <c r="U11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="V11" s="5" t="n">
-        <v>257071</v>
+        <v>256909</v>
       </c>
       <c r="W11" s="5" t="n">
         <v>0</v>
       </c>
       <c r="X11" s="5" t="n">
-        <v>50683</v>
+        <v>50356</v>
       </c>
       <c r="Y11" s="5" t="n">
-        <v>90231</v>
+        <v>90396</v>
       </c>
       <c r="Z11" s="5" t="n">
-        <v>7901</v>
+        <v>7894</v>
       </c>
       <c r="AA11" s="5" t="n">
-        <v>108256</v>
+        <v>108263</v>
       </c>
       <c r="AB11" s="5" t="n">
         <v>0</v>
@@ -1832,13 +1832,13 @@
         <v>6468</v>
       </c>
       <c r="AF11" s="5" t="n">
-        <v>108290</v>
+        <v>108442</v>
       </c>
       <c r="AG11" s="5" t="n">
         <v>27607</v>
       </c>
       <c r="AH11" s="5" t="n">
-        <v>80682</v>
+        <v>80835</v>
       </c>
       <c r="AI11" s="5" t="n">
         <v>0</v>
@@ -1872,7 +1872,7 @@
         <v>1324</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>13011</v>
+        <v>13004</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0</v>
@@ -1884,7 +1884,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>13011</v>
+        <v>13004</v>
       </c>
       <c r="N12" s="5" t="n">
         <v>0</v>
@@ -1908,13 +1908,13 @@
         <v>0</v>
       </c>
       <c r="U12" s="5" t="n">
-        <v>11687</v>
+        <v>11681</v>
       </c>
       <c r="V12" s="5" t="n">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="W12" s="5" t="n">
-        <v>2790</v>
+        <v>2789</v>
       </c>
       <c r="X12" s="5" t="n">
         <v>0</v>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="AB12" s="5" t="n">
-        <v>12145</v>
+        <v>12141</v>
       </c>
       <c r="AC12" s="5" t="n">
         <v>0</v>
@@ -1971,7 +1971,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.031</v>
+        <v>0.032</v>
       </c>
       <c r="H13" s="5" t="n">
         <v>0.533</v>
@@ -2012,7 +2012,7 @@
         <v>1</v>
       </c>
       <c r="V13" s="5" t="n">
-        <v>0.267</v>
+        <v>0.264</v>
       </c>
       <c r="W13" s="5" t="n">
         <v>1</v>
@@ -2078,53 +2078,53 @@
         <v>662.4</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>297.8</v>
+        <v>298.4</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>139.5</v>
+        <v>139.8</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>158.3</v>
+        <v>158.6</v>
       </c>
       <c r="M14" s="5" t="n">
         <v>13</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>222.7</v>
+        <v>222.5</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>263</v>
+        <v>261.9</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>198.5</v>
+        <v>197.8</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>86.40000000000001</v>
+        <v>86.2</v>
       </c>
       <c r="R14" s="5" t="n">
         <v>97.40000000000001</v>
       </c>
       <c r="S14" s="5" t="n">
-        <v>52.4</v>
+        <v>52.5</v>
       </c>
       <c r="T14" s="5" t="n">
-        <v>267.9</v>
+        <v>267.7</v>
       </c>
       <c r="U14" s="5" t="n">
         <v>11.7</v>
       </c>
       <c r="V14" s="5" t="n">
-        <v>267.9</v>
+        <v>267.7</v>
       </c>
       <c r="W14" s="5" t="inlineStr"/>
       <c r="X14" s="5" t="n">
-        <v>56.5</v>
+        <v>56.1</v>
       </c>
       <c r="Y14" s="5" t="n">
-        <v>96.2</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="Z14" s="5" t="n">
         <v>8</v>
@@ -2143,13 +2143,13 @@
         <v>11.5</v>
       </c>
       <c r="AF14" s="5" t="n">
-        <v>146.8</v>
+        <v>147</v>
       </c>
       <c r="AG14" s="5" t="n">
         <v>39.2</v>
       </c>
       <c r="AH14" s="5" t="n">
-        <v>107.6</v>
+        <v>107.8</v>
       </c>
       <c r="AI14" s="5" t="inlineStr"/>
     </row>
@@ -2177,53 +2177,53 @@
         <v>100000</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>44959</v>
+        <v>45042</v>
       </c>
       <c r="J15" s="5" t="inlineStr"/>
       <c r="K15" s="5" t="n">
-        <v>21058</v>
+        <v>21105</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>23901</v>
+        <v>23938</v>
       </c>
       <c r="M15" s="5" t="inlineStr"/>
       <c r="N15" s="5" t="n">
-        <v>33613</v>
+        <v>33584</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>39703</v>
+        <v>39539</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>29961</v>
+        <v>29853</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>13046</v>
+        <v>13017</v>
       </c>
       <c r="R15" s="5" t="n">
-        <v>14698</v>
+        <v>14701</v>
       </c>
       <c r="S15" s="5" t="n">
-        <v>7907</v>
+        <v>7930</v>
       </c>
       <c r="T15" s="5" t="n">
-        <v>40448</v>
+        <v>40413</v>
       </c>
       <c r="U15" s="5" t="inlineStr"/>
       <c r="V15" s="5" t="n">
-        <v>40448</v>
+        <v>40413</v>
       </c>
       <c r="W15" s="5" t="inlineStr"/>
       <c r="X15" s="5" t="n">
-        <v>8529</v>
+        <v>8467</v>
       </c>
       <c r="Y15" s="5" t="n">
-        <v>14526</v>
+        <v>14553</v>
       </c>
       <c r="Z15" s="5" t="n">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="AA15" s="5" t="n">
-        <v>16180</v>
+        <v>16181</v>
       </c>
       <c r="AB15" s="5" t="inlineStr"/>
       <c r="AC15" s="5" t="inlineStr"/>
@@ -2232,13 +2232,13 @@
         <v>1743</v>
       </c>
       <c r="AF15" s="5" t="n">
-        <v>22158</v>
+        <v>22195</v>
       </c>
       <c r="AG15" s="5" t="n">
         <v>5920</v>
       </c>
       <c r="AH15" s="5" t="n">
-        <v>16238</v>
+        <v>16275</v>
       </c>
       <c r="AI15" s="5" t="inlineStr"/>
     </row>
@@ -2266,18 +2266,18 @@
         <v>33.4</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>63.5</v>
+        <v>63.6</v>
       </c>
       <c r="J16" s="5" t="inlineStr"/>
       <c r="K16" s="5" t="n">
-        <v>63.5</v>
+        <v>63.6</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>63.5</v>
+        <v>63.6</v>
       </c>
       <c r="M16" s="5" t="inlineStr"/>
       <c r="N16" s="5" t="n">
-        <v>57</v>
+        <v>57.1</v>
       </c>
       <c r="O16" s="5" t="n">
         <v>46.2</v>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="W16" s="5" t="inlineStr"/>
       <c r="X16" s="5" t="n">
-        <v>26.1</v>
+        <v>25.9</v>
       </c>
       <c r="Y16" s="5" t="n">
         <v>19.3</v>
@@ -2321,7 +2321,7 @@
         <v>120.8</v>
       </c>
       <c r="AF16" s="5" t="n">
-        <v>60.1</v>
+        <v>60.2</v>
       </c>
       <c r="AG16" s="5" t="n">
         <v>69.3</v>
@@ -2355,50 +2355,50 @@
         <v>215.7</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>98</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="J17" s="5" t="inlineStr"/>
       <c r="K17" s="5" t="n">
-        <v>98</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>98</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="M17" s="5" t="inlineStr"/>
       <c r="N17" s="5" t="n">
-        <v>114.3</v>
+        <v>114.2</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>158.5</v>
+        <v>158.6</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>216.2</v>
+        <v>216.5</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>158.5</v>
+        <v>158.6</v>
       </c>
       <c r="R17" s="5" t="n">
-        <v>216.2</v>
+        <v>216.5</v>
       </c>
       <c r="S17" s="5" t="n">
-        <v>280.7</v>
+        <v>280.8</v>
       </c>
       <c r="T17" s="5" t="n">
-        <v>527.4</v>
+        <v>528.6</v>
       </c>
       <c r="U17" s="5" t="inlineStr"/>
       <c r="V17" s="5" t="n">
-        <v>527.4</v>
+        <v>528.6</v>
       </c>
       <c r="W17" s="5" t="inlineStr"/>
       <c r="X17" s="5" t="n">
-        <v>337.6</v>
+        <v>339.7</v>
       </c>
       <c r="Y17" s="5" t="n">
-        <v>462.6</v>
+        <v>462.4</v>
       </c>
       <c r="Z17" s="5" t="n">
-        <v>671.2</v>
+        <v>671.3</v>
       </c>
       <c r="AA17" s="5" t="n">
         <v>829.6</v>
@@ -2410,13 +2410,13 @@
         <v>54.2</v>
       </c>
       <c r="AF17" s="5" t="n">
-        <v>103</v>
+        <v>102.9</v>
       </c>
       <c r="AG17" s="5" t="n">
         <v>81</v>
       </c>
       <c r="AH17" s="5" t="n">
-        <v>113.5</v>
+        <v>113.3</v>
       </c>
       <c r="AI17" s="5" t="inlineStr"/>
     </row>
@@ -2442,68 +2442,70 @@
         <v>567874</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>550029</v>
+        <v>549598</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>265215</v>
-      </c>
-      <c r="I18" s="5" t="inlineStr"/>
+        <v>264993</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>101108</v>
+        <v>101310</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>114757</v>
+        <v>114910</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>13011</v>
+        <v>13004</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>166946</v>
+        <v>166764</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>209213</v>
+        <v>208349</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>166306</v>
+        <v>165727</v>
       </c>
       <c r="Q18" s="5" t="n">
-        <v>68744</v>
+        <v>68595</v>
       </c>
       <c r="R18" s="5" t="n">
-        <v>81587</v>
+        <v>81613</v>
       </c>
       <c r="S18" s="5" t="n">
-        <v>45715</v>
+        <v>45847</v>
       </c>
       <c r="T18" s="5" t="n">
-        <v>257071</v>
+        <v>256909</v>
       </c>
       <c r="U18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="V18" s="5" t="n">
-        <v>188465</v>
+        <v>189022</v>
       </c>
       <c r="W18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="X18" s="5" t="n">
-        <v>50683</v>
+        <v>50356</v>
       </c>
       <c r="Y18" s="5" t="n">
-        <v>90231</v>
+        <v>90396</v>
       </c>
       <c r="Z18" s="5" t="n">
-        <v>7901</v>
+        <v>7894</v>
       </c>
       <c r="AA18" s="5" t="n">
-        <v>108256</v>
+        <v>108263</v>
       </c>
       <c r="AB18" s="5" t="n">
-        <v>12145</v>
+        <v>12141</v>
       </c>
       <c r="AC18" s="5" t="n">
         <v>0</v>
@@ -2515,13 +2517,13 @@
         <v>6468</v>
       </c>
       <c r="AF18" s="5" t="n">
-        <v>108290</v>
+        <v>108442</v>
       </c>
       <c r="AG18" s="5" t="n">
         <v>27607</v>
       </c>
       <c r="AH18" s="5" t="n">
-        <v>80682</v>
+        <v>80835</v>
       </c>
       <c r="AI18" s="5" t="n">
         <v>0</v>
@@ -2537,59 +2539,61 @@
         <v>845.8</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>756.2</v>
+        <v>755.9</v>
       </c>
       <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="5" t="inlineStr"/>
       <c r="F19" s="5" t="n">
-        <v>756.2</v>
+        <v>755.9</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>628.5</v>
+        <v>628.2</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>669.3</v>
       </c>
-      <c r="I19" s="5" t="inlineStr"/>
+      <c r="I19" s="5" t="n">
+        <v>729</v>
+      </c>
       <c r="J19" s="5" t="inlineStr"/>
       <c r="K19" s="5" t="n">
-        <v>697.9</v>
+        <v>697.7</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>697.9</v>
+        <v>697.7</v>
       </c>
       <c r="M19" s="5" t="inlineStr"/>
       <c r="N19" s="5" t="n">
-        <v>616.8</v>
+        <v>617.1</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>592.6</v>
+        <v>591.1</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>573.8</v>
+        <v>572.7</v>
       </c>
       <c r="Q19" s="5" t="n">
         <v>771.7</v>
       </c>
       <c r="R19" s="5" t="n">
-        <v>807.8</v>
+        <v>807.9</v>
       </c>
       <c r="S19" s="5" t="n">
         <v>840.1</v>
       </c>
       <c r="T19" s="5" t="n">
-        <v>703.8</v>
+        <v>704</v>
       </c>
       <c r="U19" s="5" t="inlineStr"/>
       <c r="V19" s="5" t="n">
-        <v>685.5</v>
+        <v>685.1</v>
       </c>
       <c r="W19" s="5" t="inlineStr"/>
       <c r="X19" s="5" t="n">
-        <v>869</v>
+        <v>869.8</v>
       </c>
       <c r="Y19" s="5" t="n">
-        <v>886.5</v>
+        <v>886.4</v>
       </c>
       <c r="Z19" s="5" t="n">
         <v>934.2</v>
@@ -2604,13 +2608,13 @@
         <v>524.2</v>
       </c>
       <c r="AF19" s="5" t="n">
-        <v>553.9</v>
+        <v>553.6</v>
       </c>
       <c r="AG19" s="5" t="n">
         <v>672.3</v>
       </c>
       <c r="AH19" s="5" t="n">
-        <v>724.8</v>
+        <v>724.5</v>
       </c>
       <c r="AI19" s="5" t="inlineStr"/>
     </row>
@@ -2624,65 +2628,67 @@
         <v>671.4</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>751</v>
+        <v>751.2</v>
       </c>
       <c r="D20" s="5" t="inlineStr"/>
       <c r="E20" s="5" t="inlineStr"/>
       <c r="F20" s="5" t="n">
-        <v>751</v>
+        <v>751.2</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>875.1</v>
+        <v>874.8</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>396.2</v>
-      </c>
-      <c r="I20" s="5" t="inlineStr"/>
+        <v>395.9</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="J20" s="5" t="inlineStr"/>
       <c r="K20" s="5" t="n">
-        <v>144.9</v>
+        <v>145.2</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>164.4</v>
+        <v>164.7</v>
       </c>
       <c r="M20" s="5" t="inlineStr"/>
       <c r="N20" s="5" t="n">
-        <v>270.7</v>
+        <v>270.2</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>353</v>
+        <v>352.5</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>289.8</v>
+        <v>289.4</v>
       </c>
       <c r="Q20" s="5" t="n">
-        <v>89.09999999999999</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="R20" s="5" t="n">
         <v>101</v>
       </c>
       <c r="S20" s="5" t="n">
-        <v>54.4</v>
+        <v>54.6</v>
       </c>
       <c r="T20" s="5" t="n">
-        <v>365.3</v>
+        <v>364.9</v>
       </c>
       <c r="U20" s="5" t="inlineStr"/>
       <c r="V20" s="5" t="n">
-        <v>274.9</v>
+        <v>275.9</v>
       </c>
       <c r="W20" s="5" t="inlineStr"/>
       <c r="X20" s="5" t="n">
-        <v>58.3</v>
+        <v>57.9</v>
       </c>
       <c r="Y20" s="5" t="n">
-        <v>101.8</v>
+        <v>102</v>
       </c>
       <c r="Z20" s="5" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="AA20" s="5" t="n">
-        <v>119.6</v>
+        <v>119.7</v>
       </c>
       <c r="AB20" s="5" t="inlineStr"/>
       <c r="AC20" s="5" t="inlineStr"/>
@@ -2691,13 +2697,13 @@
         <v>12.3</v>
       </c>
       <c r="AF20" s="5" t="n">
-        <v>195.5</v>
+        <v>195.9</v>
       </c>
       <c r="AG20" s="5" t="n">
         <v>41.1</v>
       </c>
       <c r="AH20" s="5" t="n">
-        <v>111.3</v>
+        <v>111.6</v>
       </c>
       <c r="AI20" s="5" t="inlineStr"/>
     </row>
@@ -2717,13 +2723,13 @@
       </c>
       <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="n">
-        <v>17844</v>
+        <v>18275</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>303982</v>
+        <v>304204</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>228876</v>
+        <v>229224</v>
       </c>
       <c r="J21" s="5" t="n">
         <v>0</v>
@@ -2741,13 +2747,13 @@
       <c r="S21" s="5" t="inlineStr"/>
       <c r="T21" s="5" t="inlineStr"/>
       <c r="U21" s="5" t="n">
-        <v>11687</v>
+        <v>11681</v>
       </c>
       <c r="V21" s="5" t="n">
-        <v>69753</v>
+        <v>69033</v>
       </c>
       <c r="W21" s="5" t="n">
-        <v>3021</v>
+        <v>3020</v>
       </c>
       <c r="X21" s="5" t="inlineStr"/>
       <c r="Y21" s="5" t="inlineStr"/>
@@ -2769,7 +2775,7 @@
       <c r="AG21" s="5" t="inlineStr"/>
       <c r="AH21" s="5" t="inlineStr"/>
       <c r="AI21" s="5" t="n">
-        <v>6459</v>
+        <v>6443</v>
       </c>
     </row>
     <row r="22">
@@ -2784,7 +2790,7 @@
       <c r="E22" s="5" t="inlineStr"/>
       <c r="F22" s="5" t="inlineStr"/>
       <c r="G22" s="5" t="n">
-        <v>85.40000000000001</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="H22" s="5" t="n">
         <v>142.1</v>
@@ -2807,7 +2813,7 @@
         <v>18</v>
       </c>
       <c r="V22" s="5" t="n">
-        <v>283.8</v>
+        <v>284.1</v>
       </c>
       <c r="W22" s="5" t="n">
         <v>18.8</v>
@@ -2843,13 +2849,13 @@
       <c r="E23" s="5" t="inlineStr"/>
       <c r="F23" s="5" t="inlineStr"/>
       <c r="G23" s="5" t="n">
-        <v>33.817</v>
+        <v>33.857</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>9.047000000000001</v>
+        <v>9.048</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>5.076</v>
+        <v>5.086</v>
       </c>
       <c r="J23" s="5" t="inlineStr"/>
       <c r="K23" s="5" t="inlineStr"/>
@@ -2866,7 +2872,7 @@
         <v>1.5647</v>
       </c>
       <c r="V23" s="5" t="n">
-        <v>1.576</v>
+        <v>1.577</v>
       </c>
       <c r="W23" s="5" t="n">
         <v>0.0132</v>
@@ -2882,7 +2888,7 @@
       <c r="AD23" s="5" t="inlineStr"/>
       <c r="AE23" s="5" t="inlineStr"/>
       <c r="AF23" s="5" t="n">
-        <v>27.881</v>
+        <v>27.895</v>
       </c>
       <c r="AG23" s="5" t="inlineStr"/>
       <c r="AH23" s="5" t="inlineStr"/>
@@ -2902,13 +2908,13 @@
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="n">
-        <v>528</v>
+        <v>540</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>33599</v>
+        <v>33620</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>45092</v>
+        <v>45065</v>
       </c>
       <c r="J24" s="5" t="inlineStr"/>
       <c r="K24" s="5" t="inlineStr"/>
@@ -2922,13 +2928,13 @@
       <c r="S24" s="5" t="inlineStr"/>
       <c r="T24" s="5" t="inlineStr"/>
       <c r="U24" s="5" t="n">
-        <v>7470</v>
+        <v>7465</v>
       </c>
       <c r="V24" s="5" t="n">
-        <v>44266</v>
+        <v>43771</v>
       </c>
       <c r="W24" s="5" t="n">
-        <v>229183</v>
+        <v>229101</v>
       </c>
       <c r="X24" s="5" t="inlineStr"/>
       <c r="Y24" s="5" t="inlineStr"/>
@@ -2946,7 +2952,7 @@
       <c r="AG24" s="5" t="inlineStr"/>
       <c r="AH24" s="5" t="inlineStr"/>
       <c r="AI24" s="5" t="n">
-        <v>1809</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="25">
@@ -2959,67 +2965,67 @@
         <v>4534</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>40794</v>
+        <v>40904</v>
       </c>
       <c r="D25" s="5" t="inlineStr"/>
       <c r="E25" s="5" t="inlineStr"/>
       <c r="F25" s="5" t="n">
-        <v>40701</v>
+        <v>40811</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>99504</v>
+        <v>99751</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>158234</v>
+        <v>158323</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>44089</v>
+        <v>44020</v>
       </c>
       <c r="J25" s="5" t="inlineStr"/>
       <c r="K25" s="5" t="n">
-        <v>1806</v>
+        <v>1810</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>2050</v>
+        <v>2053</v>
       </c>
       <c r="M25" s="5" t="inlineStr"/>
       <c r="N25" s="5" t="n">
-        <v>15035</v>
+        <v>14967</v>
       </c>
       <c r="O25" s="5" t="n">
-        <v>31925</v>
+        <v>32053</v>
       </c>
       <c r="P25" s="5" t="n">
-        <v>34960</v>
+        <v>35021</v>
       </c>
       <c r="Q25" s="5" t="n">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="R25" s="5" t="n">
         <v>1812</v>
       </c>
       <c r="S25" s="5" t="n">
-        <v>1119</v>
+        <v>1122</v>
       </c>
       <c r="T25" s="5" t="n">
-        <v>56973</v>
+        <v>56964</v>
       </c>
       <c r="U25" s="5" t="inlineStr"/>
       <c r="V25" s="5" t="n">
-        <v>72600</v>
+        <v>72541</v>
       </c>
       <c r="W25" s="5" t="inlineStr"/>
       <c r="X25" s="5" t="n">
-        <v>1077</v>
+        <v>1069</v>
       </c>
       <c r="Y25" s="5" t="n">
-        <v>3612</v>
+        <v>3619</v>
       </c>
       <c r="Z25" s="5" t="n">
         <v>305</v>
       </c>
       <c r="AA25" s="5" t="n">
-        <v>9489</v>
+        <v>9490</v>
       </c>
       <c r="AB25" s="5" t="inlineStr"/>
       <c r="AC25" s="5" t="inlineStr"/>
@@ -3028,13 +3034,13 @@
         <v>135</v>
       </c>
       <c r="AF25" s="5" t="n">
-        <v>13960</v>
+        <v>13985</v>
       </c>
       <c r="AG25" s="5" t="n">
         <v>586</v>
       </c>
       <c r="AH25" s="5" t="n">
-        <v>1416</v>
+        <v>1419</v>
       </c>
       <c r="AI25" s="5" t="inlineStr"/>
     </row>
@@ -3076,30 +3082,30 @@
         <v>19</v>
       </c>
       <c r="O26" s="5" t="n">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="P26" s="5" t="n">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="Q26" s="5" t="n">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="R26" s="5" t="n">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="S26" s="5" t="n">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="T26" s="5" t="n">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="U26" s="5" t="inlineStr"/>
       <c r="V26" s="5" t="n">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="W26" s="5" t="inlineStr"/>
       <c r="X26" s="5" t="n">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="Y26" s="5" t="n">
         <v>418</v>
@@ -3240,33 +3246,33 @@
         <v>716</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="J28" s="5" t="inlineStr"/>
       <c r="K28" s="5" t="n">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="M28" s="5" t="inlineStr"/>
       <c r="N28" s="5" t="n">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="O28" s="5" t="n">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="P28" s="5" t="n">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="Q28" s="5" t="n">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="R28" s="5" t="n">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="S28" s="5" t="n">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="T28" s="5" t="n">
         <v>789</v>
@@ -3295,13 +3301,13 @@
         <v>39</v>
       </c>
       <c r="AF28" s="5" t="n">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="AG28" s="5" t="n">
         <v>84</v>
       </c>
       <c r="AH28" s="5" t="n">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AI28" s="5" t="inlineStr"/>
     </row>
@@ -3329,44 +3335,44 @@
         <v>1.8</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>0.044</v>
+        <v>0.043</v>
       </c>
       <c r="J29" s="5" t="inlineStr"/>
       <c r="K29" s="5" t="n">
-        <v>0.044</v>
+        <v>0.043</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>0.044</v>
+        <v>0.043</v>
       </c>
       <c r="M29" s="5" t="inlineStr"/>
       <c r="N29" s="5" t="n">
-        <v>0.119</v>
+        <v>0.116</v>
       </c>
       <c r="O29" s="5" t="n">
-        <v>0.244</v>
+        <v>0.238</v>
       </c>
       <c r="P29" s="5" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
       <c r="Q29" s="5" t="n">
-        <v>0.244</v>
+        <v>0.238</v>
       </c>
       <c r="R29" s="5" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
       <c r="S29" s="5" t="n">
-        <v>1.778</v>
+        <v>1.779</v>
       </c>
       <c r="T29" s="5" t="n">
-        <v>3.274</v>
+        <v>3.277</v>
       </c>
       <c r="U29" s="5" t="inlineStr"/>
       <c r="V29" s="5" t="n">
-        <v>3.274</v>
+        <v>3.277</v>
       </c>
       <c r="W29" s="5" t="inlineStr"/>
       <c r="X29" s="5" t="n">
-        <v>2.279</v>
+        <v>2.295</v>
       </c>
       <c r="Y29" s="5" t="n">
         <v>2.892</v>
@@ -3384,13 +3390,13 @@
         <v>0.001</v>
       </c>
       <c r="AF29" s="5" t="n">
-        <v>0.046</v>
+        <v>0.045</v>
       </c>
       <c r="AG29" s="5" t="n">
         <v>0.018</v>
       </c>
       <c r="AH29" s="5" t="n">
-        <v>0.056</v>
+        <v>0.055</v>
       </c>
       <c r="AI29" s="5" t="inlineStr"/>
     </row>
@@ -3738,13 +3744,13 @@
         <v>117.8</v>
       </c>
       <c r="R4" s="9" t="n">
-        <v>221.6</v>
+        <v>221.7</v>
       </c>
       <c r="S4" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T4" s="9" t="n">
-        <v>103.8</v>
+        <v>103.9</v>
       </c>
       <c r="U4" s="9" t="n">
         <v>117.8</v>
@@ -3753,7 +3759,7 @@
         <v>0</v>
       </c>
       <c r="W4" s="9" t="n">
-        <v>107.2</v>
+        <v>107.1</v>
       </c>
       <c r="X4" s="9" t="n">
         <v>0</v>
@@ -3768,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="AB4" s="9" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AC4" s="9" t="n">
         <v>0</v>
@@ -3874,13 +3880,13 @@
         <v>1342.1</v>
       </c>
       <c r="R5" s="10" t="n">
-        <v>2524.6</v>
+        <v>2525.4</v>
       </c>
       <c r="S5" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T5" s="10" t="n">
-        <v>1182.5</v>
+        <v>1183.3</v>
       </c>
       <c r="U5" s="10" t="n">
         <v>1342.1</v>
@@ -3889,7 +3895,7 @@
         <v>0</v>
       </c>
       <c r="W5" s="10" t="n">
-        <v>1221</v>
+        <v>1219.7</v>
       </c>
       <c r="X5" s="9" t="n">
         <v>0</v>
@@ -4010,13 +4016,13 @@
         <v>931.5</v>
       </c>
       <c r="R6" s="10" t="n">
-        <v>1752.1</v>
+        <v>1752.7</v>
       </c>
       <c r="S6" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T6" s="9" t="n">
-        <v>820.7</v>
+        <v>821.2</v>
       </c>
       <c r="U6" s="9" t="n">
         <v>931.5</v>
@@ -4025,7 +4031,7 @@
         <v>0</v>
       </c>
       <c r="W6" s="9" t="n">
-        <v>847.4</v>
+        <v>846.5</v>
       </c>
       <c r="X6" s="9" t="n">
         <v>0</v>
@@ -4146,13 +4152,13 @@
         <v>3864.8</v>
       </c>
       <c r="R7" s="10" t="n">
-        <v>7269.9</v>
+        <v>7272.2</v>
       </c>
       <c r="S7" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T7" s="10" t="n">
-        <v>3405.1</v>
+        <v>3407.4</v>
       </c>
       <c r="U7" s="10" t="n">
         <v>3864.8</v>
@@ -4161,19 +4167,19 @@
         <v>0</v>
       </c>
       <c r="W7" s="10" t="n">
-        <v>3516.1</v>
+        <v>3512.2</v>
       </c>
       <c r="X7" s="9" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Y7" s="9" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z7" s="9" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA7" s="9" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AB7" s="9" t="n">
         <v>-0</v>
@@ -4282,13 +4288,13 @@
         <v>8824.700000000001</v>
       </c>
       <c r="R8" s="10" t="n">
-        <v>16599.8</v>
+        <v>16605</v>
       </c>
       <c r="S8" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T8" s="10" t="n">
-        <v>7775.1</v>
+        <v>7780.3</v>
       </c>
       <c r="U8" s="10" t="n">
         <v>8824.700000000001</v>
@@ -4297,7 +4303,7 @@
         <v>0</v>
       </c>
       <c r="W8" s="10" t="n">
-        <v>8028.5</v>
+        <v>8019.6</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>0</v>
@@ -4418,13 +4424,13 @@
         <v>9584.4</v>
       </c>
       <c r="R9" s="10" t="n">
-        <v>18028.8</v>
+        <v>18034.5</v>
       </c>
       <c r="S9" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T9" s="10" t="n">
-        <v>8444.4</v>
+        <v>8450.1</v>
       </c>
       <c r="U9" s="10" t="n">
         <v>9584.4</v>
@@ -4433,7 +4439,7 @@
         <v>0</v>
       </c>
       <c r="W9" s="10" t="n">
-        <v>8719.700000000001</v>
+        <v>8710</v>
       </c>
       <c r="X9" s="9" t="n">
         <v>0</v>
@@ -4554,13 +4560,13 @@
         <v>9352</v>
       </c>
       <c r="R10" s="10" t="n">
-        <v>17591.6</v>
+        <v>17597.1</v>
       </c>
       <c r="S10" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T10" s="10" t="n">
-        <v>8239.6</v>
+        <v>8245.1</v>
       </c>
       <c r="U10" s="10" t="n">
         <v>9352</v>
@@ -4569,10 +4575,10 @@
         <v>0</v>
       </c>
       <c r="W10" s="10" t="n">
-        <v>8508.200000000001</v>
+        <v>8498.799999999999</v>
       </c>
       <c r="X10" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="Y10" s="9" t="n">
         <v>0</v>
@@ -4690,31 +4696,31 @@
         <v>10500.2</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>19751.1</v>
+        <v>19757.6</v>
       </c>
       <c r="S11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>9251.1</v>
+        <v>9257.4</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>10500</v>
+        <v>10500.2</v>
       </c>
       <c r="V11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W11" s="10" t="n">
-        <v>9552.799999999999</v>
+        <v>9542.200000000001</v>
       </c>
       <c r="X11" s="9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="Y11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="Z11" s="9" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="9" t="n">
         <v>0</v>
@@ -4759,13 +4765,13 @@
         <v>0.1</v>
       </c>
       <c r="AO11" s="10" t="n">
-        <v>10499.8</v>
+        <v>10500</v>
       </c>
       <c r="AP11" s="9" t="n">
         <v>525</v>
       </c>
       <c r="AQ11" s="10" t="n">
-        <v>9974.799999999999</v>
+        <v>9975</v>
       </c>
       <c r="AR11" s="9" t="n">
         <v>0</v>
@@ -4826,31 +4832,31 @@
         <v>13390.2</v>
       </c>
       <c r="R12" s="10" t="n">
-        <v>25184.1</v>
+        <v>25195.5</v>
       </c>
       <c r="S12" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T12" s="10" t="n">
-        <v>11795.9</v>
+        <v>11805.4</v>
       </c>
       <c r="U12" s="10" t="n">
-        <v>13388.3</v>
+        <v>13390.1</v>
       </c>
       <c r="V12" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W12" s="10" t="n">
-        <v>12182.1</v>
+        <v>12168.6</v>
       </c>
       <c r="X12" s="9" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="9" t="n">
         <v>0</v>
       </c>
       <c r="Z12" s="9" t="n">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="9" t="n">
         <v>0</v>
@@ -4895,13 +4901,13 @@
         <v>0</v>
       </c>
       <c r="AO12" s="10" t="n">
-        <v>13388.3</v>
+        <v>13390.1</v>
       </c>
       <c r="AP12" s="9" t="n">
         <v>1.9</v>
       </c>
       <c r="AQ12" s="10" t="n">
-        <v>13386.3</v>
+        <v>13388.2</v>
       </c>
       <c r="AR12" s="9" t="n">
         <v>0</v>
@@ -4962,31 +4968,31 @@
         <v>15698.1</v>
       </c>
       <c r="R13" s="10" t="n">
-        <v>29494.2</v>
+        <v>29537.4</v>
       </c>
       <c r="S13" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T13" s="10" t="n">
-        <v>13814.6</v>
+        <v>13839.8</v>
       </c>
       <c r="U13" s="10" t="n">
-        <v>15679.6</v>
+        <v>15697.6</v>
       </c>
       <c r="V13" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W13" s="10" t="n">
-        <v>14281.8</v>
+        <v>14265.9</v>
       </c>
       <c r="X13" s="9" t="n">
-        <v>56.3</v>
+        <v>1.3</v>
       </c>
       <c r="Y13" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="9" t="n">
-        <v>18.5</v>
+        <v>0.4</v>
       </c>
       <c r="AA13" s="9" t="n">
         <v>0</v>
@@ -5031,13 +5037,13 @@
         <v>0</v>
       </c>
       <c r="AO13" s="10" t="n">
-        <v>15679.6</v>
+        <v>15697.6</v>
       </c>
       <c r="AP13" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AQ13" s="10" t="n">
-        <v>15679.6</v>
+        <v>15697.6</v>
       </c>
       <c r="AR13" s="9" t="n">
         <v>0</v>
@@ -5098,34 +5104,34 @@
         <v>16099.2</v>
       </c>
       <c r="R14" s="10" t="n">
-        <v>29996</v>
+        <v>30271.1</v>
       </c>
       <c r="S14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T14" s="10" t="n">
-        <v>14049.6</v>
+        <v>14183.5</v>
       </c>
       <c r="U14" s="10" t="n">
-        <v>15946.3</v>
+        <v>16087.5</v>
       </c>
       <c r="V14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W14" s="10" t="n">
-        <v>14646.6</v>
+        <v>14630.4</v>
       </c>
       <c r="X14" s="9" t="n">
-        <v>464.7</v>
+        <v>35.4</v>
       </c>
       <c r="Y14" s="9" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="Z14" s="9" t="n">
-        <v>152.7</v>
+        <v>11.7</v>
       </c>
       <c r="AA14" s="9" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="AB14" s="9" t="n">
         <v>-0</v>
@@ -5167,13 +5173,13 @@
         <v>0</v>
       </c>
       <c r="AO14" s="10" t="n">
-        <v>15946.3</v>
+        <v>16087.5</v>
       </c>
       <c r="AP14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AQ14" s="10" t="n">
-        <v>15946.3</v>
+        <v>16087.5</v>
       </c>
       <c r="AR14" s="9" t="n">
         <v>0</v>
@@ -5234,37 +5240,37 @@
         <v>15103.8</v>
       </c>
       <c r="R15" s="10" t="n">
-        <v>26281</v>
+        <v>27860.9</v>
       </c>
       <c r="S15" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T15" s="10" t="n">
-        <v>12309.6</v>
+        <v>13054.3</v>
       </c>
       <c r="U15" s="10" t="n">
-        <v>13971.4</v>
+        <v>14806.7</v>
       </c>
       <c r="V15" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W15" s="10" t="n">
-        <v>13740.3</v>
-      </c>
-      <c r="X15" s="10" t="n">
-        <v>3443.6</v>
+        <v>13725.8</v>
+      </c>
+      <c r="X15" s="9" t="n">
+        <v>902.5</v>
       </c>
       <c r="Y15" s="9" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="Z15" s="10" t="n">
-        <v>1131.5</v>
+        <v>0</v>
+      </c>
+      <c r="Z15" s="9" t="n">
+        <v>297.1</v>
       </c>
       <c r="AA15" s="9" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="AB15" s="9" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AC15" s="9" t="n">
         <v>0</v>
@@ -5303,13 +5309,13 @@
         <v>0</v>
       </c>
       <c r="AO15" s="10" t="n">
-        <v>13971.4</v>
+        <v>14806.7</v>
       </c>
       <c r="AP15" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AQ15" s="10" t="n">
-        <v>13971.4</v>
+        <v>14806.7</v>
       </c>
       <c r="AR15" s="9" t="n">
         <v>0</v>
@@ -5370,37 +5376,37 @@
         <v>14913.7</v>
       </c>
       <c r="R16" s="10" t="n">
-        <v>16538.1</v>
+        <v>17880.3</v>
       </c>
       <c r="S16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T16" s="10" t="n">
-        <v>7746.2</v>
+        <v>8377.799999999999</v>
       </c>
       <c r="U16" s="10" t="n">
-        <v>8791.9</v>
+        <v>9502.5</v>
       </c>
       <c r="V16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W16" s="10" t="n">
-        <v>13563.9</v>
+        <v>13552.9</v>
       </c>
       <c r="X16" s="10" t="n">
-        <v>18616.5</v>
+        <v>16435.2</v>
       </c>
       <c r="Y16" s="9" t="n">
-        <v>9.6</v>
+        <v>0.4</v>
       </c>
       <c r="Z16" s="10" t="n">
-        <v>6117.1</v>
+        <v>5411</v>
       </c>
       <c r="AA16" s="9" t="n">
-        <v>4.7</v>
+        <v>0.2</v>
       </c>
       <c r="AB16" s="9" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AC16" s="9" t="n">
         <v>0</v>
@@ -5439,13 +5445,13 @@
         <v>0</v>
       </c>
       <c r="AO16" s="10" t="n">
-        <v>8791.9</v>
+        <v>9502.5</v>
       </c>
       <c r="AP16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AQ16" s="10" t="n">
-        <v>8791.9</v>
+        <v>9502.5</v>
       </c>
       <c r="AR16" s="9" t="n">
         <v>0</v>
@@ -5506,34 +5512,34 @@
         <v>14837.4</v>
       </c>
       <c r="R17" s="10" t="n">
-        <v>4021.8</v>
+        <v>1644</v>
       </c>
       <c r="S17" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T17" s="10" t="n">
-        <v>1883.8</v>
-      </c>
-      <c r="U17" s="10" t="n">
-        <v>2138.1</v>
+      <c r="T17" s="9" t="n">
+        <v>770.3</v>
+      </c>
+      <c r="U17" s="9" t="n">
+        <v>873.7</v>
       </c>
       <c r="V17" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W17" s="10" t="n">
-        <v>13476.2</v>
+        <v>13481.8</v>
       </c>
       <c r="X17" s="10" t="n">
-        <v>38573.4</v>
+        <v>42406.4</v>
       </c>
       <c r="Y17" s="9" t="n">
-        <v>50.5</v>
+        <v>4.3</v>
       </c>
       <c r="Z17" s="10" t="n">
-        <v>12674.5</v>
+        <v>13961.6</v>
       </c>
       <c r="AA17" s="9" t="n">
-        <v>24.8</v>
+        <v>2.1</v>
       </c>
       <c r="AB17" s="9" t="n">
         <v>0</v>
@@ -5574,14 +5580,14 @@
       <c r="AN17" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AO17" s="10" t="n">
-        <v>2138.1</v>
+      <c r="AO17" s="9" t="n">
+        <v>873.7</v>
       </c>
       <c r="AP17" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AQ17" s="10" t="n">
-        <v>2138.1</v>
+      <c r="AQ17" s="9" t="n">
+        <v>873.7</v>
       </c>
       <c r="AR17" s="9" t="n">
         <v>0</v>
@@ -5642,37 +5648,37 @@
         <v>14768.3</v>
       </c>
       <c r="R18" s="9" t="n">
-        <v>538</v>
+        <v>61.9</v>
       </c>
       <c r="S18" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T18" s="9" t="n">
-        <v>252</v>
+        <v>29</v>
       </c>
       <c r="U18" s="9" t="n">
-        <v>286</v>
+        <v>32.9</v>
       </c>
       <c r="V18" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W18" s="10" t="n">
-        <v>13317.8</v>
+        <v>13401.7</v>
       </c>
       <c r="X18" s="10" t="n">
-        <v>43680</v>
+        <v>44692.4</v>
       </c>
       <c r="Y18" s="9" t="n">
-        <v>264.4</v>
+        <v>43.1</v>
       </c>
       <c r="Z18" s="10" t="n">
-        <v>14352.5</v>
+        <v>14714.2</v>
       </c>
       <c r="AA18" s="9" t="n">
-        <v>129.7</v>
+        <v>21.2</v>
       </c>
       <c r="AB18" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AC18" s="9" t="n">
         <v>0</v>
@@ -5711,13 +5717,13 @@
         <v>0</v>
       </c>
       <c r="AO18" s="9" t="n">
-        <v>286</v>
+        <v>32.9</v>
       </c>
       <c r="AP18" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AQ18" s="9" t="n">
-        <v>286</v>
+        <v>32.9</v>
       </c>
       <c r="AR18" s="9" t="n">
         <v>0</v>
@@ -5778,52 +5784,52 @@
         <v>14697.6</v>
       </c>
       <c r="R19" s="9" t="n">
-        <v>63.9</v>
+        <v>2.2</v>
       </c>
       <c r="S19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T19" s="9" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="U19" s="9" t="n">
-        <v>34</v>
+        <v>1.2</v>
       </c>
       <c r="V19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W19" s="10" t="n">
-        <v>12772.2</v>
+        <v>13166.2</v>
       </c>
       <c r="X19" s="10" t="n">
-        <v>42621.7</v>
-      </c>
-      <c r="Y19" s="10" t="n">
-        <v>1341.9</v>
+        <v>44001.7</v>
+      </c>
+      <c r="Y19" s="9" t="n">
+        <v>425.6</v>
       </c>
       <c r="Z19" s="10" t="n">
-        <v>14004.7</v>
+        <v>14486.8</v>
       </c>
       <c r="AA19" s="9" t="n">
-        <v>658.3</v>
+        <v>209.6</v>
       </c>
       <c r="AB19" s="9" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="AC19" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AD19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE19" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AF19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG19" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AH19" s="9" t="n">
         <v>0</v>
@@ -5847,13 +5853,13 @@
         <v>0</v>
       </c>
       <c r="AO19" s="9" t="n">
-        <v>34</v>
+        <v>1.2</v>
       </c>
       <c r="AP19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AQ19" s="9" t="n">
-        <v>34</v>
+        <v>1.2</v>
       </c>
       <c r="AR19" s="9" t="n">
         <v>0</v>
@@ -5914,52 +5920,52 @@
         <v>14627.8</v>
       </c>
       <c r="R20" s="9" t="n">
-        <v>7.5</v>
+        <v>0.1</v>
       </c>
       <c r="S20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T20" s="9" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="U20" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W20" s="10" t="n">
-        <v>10658.7</v>
+        <v>11604.6</v>
       </c>
       <c r="X20" s="10" t="n">
-        <v>35643</v>
+        <v>38785.7</v>
       </c>
       <c r="Y20" s="10" t="n">
-        <v>5932</v>
+        <v>3773</v>
       </c>
       <c r="Z20" s="10" t="n">
-        <v>11711.7</v>
+        <v>12769.5</v>
       </c>
       <c r="AA20" s="10" t="n">
-        <v>2910.1</v>
+        <v>1858</v>
       </c>
       <c r="AB20" s="9" t="n">
-        <v>1.7</v>
+        <v>0.2</v>
       </c>
       <c r="AC20" s="9" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="AD20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE20" s="9" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="AF20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG20" s="9" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="AH20" s="9" t="n">
         <v>0</v>
@@ -5983,13 +5989,13 @@
         <v>0</v>
       </c>
       <c r="AO20" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AP20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AQ20" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AR20" s="9" t="n">
         <v>0</v>
@@ -6050,52 +6056,52 @@
         <v>14563.6</v>
       </c>
       <c r="R21" s="9" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="S21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="T21" s="9" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="U21" s="9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="V21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="W21" s="10" t="n">
-        <v>5719.3</v>
+        <v>5372.2</v>
       </c>
       <c r="X21" s="10" t="n">
-        <v>19130.7</v>
+        <v>17955.4</v>
       </c>
       <c r="Y21" s="10" t="n">
-        <v>16855.8</v>
+        <v>17566.4</v>
       </c>
       <c r="Z21" s="10" t="n">
-        <v>6286</v>
+        <v>5911.5</v>
       </c>
       <c r="AA21" s="10" t="n">
-        <v>8269.1</v>
+        <v>8650.6</v>
       </c>
       <c r="AB21" s="9" t="n">
-        <v>6.9</v>
+        <v>1.3</v>
       </c>
       <c r="AC21" s="9" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="AD21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE21" s="9" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="AF21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG21" s="9" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="AH21" s="9" t="n">
         <v>0</v>
@@ -6119,13 +6125,13 @@
         <v>0</v>
       </c>
       <c r="AO21" s="9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AP21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AQ21" s="9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AR21" s="9" t="n">
         <v>0</v>
@@ -6186,7 +6192,7 @@
         <v>14511</v>
       </c>
       <c r="R22" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="S22" s="9" t="n">
         <v>0</v>
@@ -6195,43 +6201,43 @@
         <v>0</v>
       </c>
       <c r="U22" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="V22" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="W22" s="10" t="n">
-        <v>1656</v>
+      <c r="W22" s="9" t="n">
+        <v>839.2</v>
       </c>
       <c r="X22" s="10" t="n">
-        <v>5539.5</v>
+        <v>2804.9</v>
       </c>
       <c r="Y22" s="10" t="n">
-        <v>25805.2</v>
-      </c>
-      <c r="Z22" s="10" t="n">
-        <v>1820.2</v>
+        <v>27575.4</v>
+      </c>
+      <c r="Z22" s="9" t="n">
+        <v>923.5</v>
       </c>
       <c r="AA22" s="10" t="n">
-        <v>12659.5</v>
+        <v>13579.5</v>
       </c>
       <c r="AB22" s="9" t="n">
-        <v>28</v>
+        <v>7.2</v>
       </c>
       <c r="AC22" s="9" t="n">
-        <v>3.3</v>
+        <v>0.8</v>
       </c>
       <c r="AD22" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE22" s="9" t="n">
-        <v>3.3</v>
+        <v>0.8</v>
       </c>
       <c r="AF22" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG22" s="9" t="n">
-        <v>3.3</v>
+        <v>0.8</v>
       </c>
       <c r="AH22" s="9" t="n">
         <v>0</v>
@@ -6255,13 +6261,13 @@
         <v>0</v>
       </c>
       <c r="AO22" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AP22" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AQ22" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AR22" s="9" t="n">
         <v>0</v>
@@ -6337,37 +6343,37 @@
         <v>0</v>
       </c>
       <c r="W23" s="9" t="n">
-        <v>347.6</v>
-      </c>
-      <c r="X23" s="10" t="n">
-        <v>1162.6</v>
+        <v>88.40000000000001</v>
+      </c>
+      <c r="X23" s="9" t="n">
+        <v>295.5</v>
       </c>
       <c r="Y23" s="10" t="n">
-        <v>28481</v>
+        <v>29111.3</v>
       </c>
       <c r="Z23" s="9" t="n">
-        <v>382</v>
+        <v>97.3</v>
       </c>
       <c r="AA23" s="10" t="n">
-        <v>13972.2</v>
+        <v>14335.9</v>
       </c>
       <c r="AB23" s="9" t="n">
-        <v>111.5</v>
+        <v>39.3</v>
       </c>
       <c r="AC23" s="9" t="n">
-        <v>9.5</v>
+        <v>2.8</v>
       </c>
       <c r="AD23" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE23" s="9" t="n">
-        <v>9.5</v>
+        <v>2.8</v>
       </c>
       <c r="AF23" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG23" s="9" t="n">
-        <v>9.5</v>
+        <v>2.8</v>
       </c>
       <c r="AH23" s="9" t="n">
         <v>0</v>
@@ -6473,37 +6479,37 @@
         <v>0</v>
       </c>
       <c r="W24" s="9" t="n">
-        <v>66.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="X24" s="9" t="n">
-        <v>223.3</v>
+        <v>29.4</v>
       </c>
       <c r="Y24" s="10" t="n">
-        <v>28274.6</v>
+        <v>28785.2</v>
       </c>
       <c r="Z24" s="9" t="n">
-        <v>73.40000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AA24" s="10" t="n">
-        <v>13870.9</v>
+        <v>14175.3</v>
       </c>
       <c r="AB24" s="9" t="n">
-        <v>432.2</v>
+        <v>209.4</v>
       </c>
       <c r="AC24" s="9" t="n">
-        <v>27.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AD24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE24" s="9" t="n">
-        <v>27.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AF24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG24" s="9" t="n">
-        <v>27.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AH24" s="9" t="n">
         <v>0</v>
@@ -6609,37 +6615,37 @@
         <v>0</v>
       </c>
       <c r="W25" s="9" t="n">
-        <v>12.6</v>
+        <v>0.9</v>
       </c>
       <c r="X25" s="9" t="n">
-        <v>42</v>
+        <v>2.9</v>
       </c>
       <c r="Y25" s="10" t="n">
-        <v>25775.1</v>
+        <v>26823.7</v>
       </c>
       <c r="Z25" s="9" t="n">
-        <v>13.8</v>
+        <v>1</v>
       </c>
       <c r="AA25" s="10" t="n">
-        <v>12644.8</v>
+        <v>13209.4</v>
       </c>
       <c r="AB25" s="10" t="n">
-        <v>1552.4</v>
+        <v>1046.8</v>
       </c>
       <c r="AC25" s="9" t="n">
-        <v>79.90000000000001</v>
+        <v>33.8</v>
       </c>
       <c r="AD25" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE25" s="9" t="n">
-        <v>79.90000000000001</v>
+        <v>33.8</v>
       </c>
       <c r="AF25" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG25" s="9" t="n">
-        <v>79.90000000000001</v>
+        <v>33.8</v>
       </c>
       <c r="AH25" s="9" t="n">
         <v>0</v>
@@ -6745,37 +6751,37 @@
         <v>0</v>
       </c>
       <c r="W26" s="9" t="n">
-        <v>2.4</v>
+        <v>0.1</v>
       </c>
       <c r="X26" s="9" t="n">
-        <v>7.9</v>
+        <v>0.3</v>
       </c>
       <c r="Y26" s="10" t="n">
-        <v>19236.2</v>
+        <v>20118.7</v>
       </c>
       <c r="Z26" s="9" t="n">
-        <v>2.6</v>
+        <v>0.1</v>
       </c>
       <c r="AA26" s="10" t="n">
-        <v>9436.9</v>
+        <v>9907.5</v>
       </c>
       <c r="AB26" s="10" t="n">
-        <v>4540.1</v>
+        <v>4185</v>
       </c>
       <c r="AC26" s="9" t="n">
-        <v>229.9</v>
+        <v>116.9</v>
       </c>
       <c r="AD26" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE26" s="9" t="n">
-        <v>229.9</v>
+        <v>116.9</v>
       </c>
       <c r="AF26" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG26" s="9" t="n">
-        <v>229.9</v>
+        <v>116.9</v>
       </c>
       <c r="AH26" s="9" t="n">
         <v>0</v>
@@ -6881,37 +6887,37 @@
         <v>0</v>
       </c>
       <c r="W27" s="9" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="X27" s="9" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="Y27" s="10" t="n">
-        <v>9776.9</v>
+        <v>8792.799999999999</v>
       </c>
       <c r="Z27" s="9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AA27" s="10" t="n">
-        <v>4796.4</v>
+        <v>4330.1</v>
       </c>
       <c r="AB27" s="10" t="n">
-        <v>8796.200000000001</v>
+        <v>9514.4</v>
       </c>
       <c r="AC27" s="9" t="n">
-        <v>650.9</v>
+        <v>399.5</v>
       </c>
       <c r="AD27" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE27" s="9" t="n">
-        <v>650.9</v>
+        <v>399.5</v>
       </c>
       <c r="AF27" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG27" s="9" t="n">
-        <v>650.8</v>
+        <v>399.4</v>
       </c>
       <c r="AH27" s="9" t="n">
         <v>0.1</v>
@@ -7017,40 +7023,40 @@
         <v>0</v>
       </c>
       <c r="W28" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="X28" s="9" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="Y28" s="10" t="n">
-        <v>3304.7</v>
+        <v>2184.6</v>
       </c>
       <c r="Z28" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AA28" s="10" t="n">
-        <v>1621.2</v>
+        <v>1075.8</v>
       </c>
       <c r="AB28" s="10" t="n">
-        <v>10729</v>
+        <v>11712.6</v>
       </c>
       <c r="AC28" s="10" t="n">
-        <v>1722.9</v>
+        <v>1284.8</v>
       </c>
       <c r="AD28" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE28" s="10" t="n">
-        <v>1722.9</v>
+        <v>1284.8</v>
       </c>
       <c r="AF28" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG28" s="10" t="n">
-        <v>1721.8</v>
+        <v>1284</v>
       </c>
       <c r="AH28" s="9" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="AI28" s="9" t="n">
         <v>0</v>
@@ -7156,37 +7162,37 @@
         <v>0</v>
       </c>
       <c r="X29" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="Y29" s="9" t="n">
-        <v>898.3</v>
+        <v>427.6</v>
       </c>
       <c r="Z29" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AA29" s="9" t="n">
-        <v>440.7</v>
+        <v>210.5</v>
       </c>
       <c r="AB29" s="10" t="n">
-        <v>9274</v>
+        <v>9911.6</v>
       </c>
       <c r="AC29" s="10" t="n">
-        <v>3955.2</v>
+        <v>3547.9</v>
       </c>
       <c r="AD29" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE29" s="10" t="n">
-        <v>3955.2</v>
+        <v>3547.9</v>
       </c>
       <c r="AF29" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG29" s="10" t="n">
-        <v>3945.9</v>
+        <v>3539.5</v>
       </c>
       <c r="AH29" s="9" t="n">
-        <v>9.300000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AI29" s="9" t="n">
         <v>0</v>
@@ -7295,34 +7301,34 @@
         <v>0</v>
       </c>
       <c r="Y30" s="9" t="n">
-        <v>225.5</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="Z30" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AA30" s="9" t="n">
-        <v>110.6</v>
+        <v>38.6</v>
       </c>
       <c r="AB30" s="10" t="n">
-        <v>5867.2</v>
+        <v>5846.7</v>
       </c>
       <c r="AC30" s="10" t="n">
-        <v>7095.2</v>
+        <v>7187.7</v>
       </c>
       <c r="AD30" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE30" s="10" t="n">
-        <v>7095.2</v>
+        <v>7187.7</v>
       </c>
       <c r="AF30" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG30" s="10" t="n">
-        <v>7037.3</v>
+        <v>7129.1</v>
       </c>
       <c r="AH30" s="9" t="n">
-        <v>57.8</v>
+        <v>58.6</v>
       </c>
       <c r="AI30" s="9" t="n">
         <v>0</v>
@@ -7431,34 +7437,34 @@
         <v>0</v>
       </c>
       <c r="Y31" s="9" t="n">
-        <v>55.9</v>
+        <v>14.3</v>
       </c>
       <c r="Z31" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AA31" s="9" t="n">
-        <v>27.4</v>
+        <v>7</v>
       </c>
       <c r="AB31" s="10" t="n">
-        <v>2793.3</v>
+        <v>2385.8</v>
       </c>
       <c r="AC31" s="10" t="n">
-        <v>9786.299999999999</v>
+        <v>10214.3</v>
       </c>
       <c r="AD31" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE31" s="10" t="n">
-        <v>9786.299999999999</v>
+        <v>10214.3</v>
       </c>
       <c r="AF31" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG31" s="10" t="n">
-        <v>9512.700000000001</v>
+        <v>9928.700000000001</v>
       </c>
       <c r="AH31" s="9" t="n">
-        <v>273.2</v>
+        <v>285.2</v>
       </c>
       <c r="AI31" s="9" t="n">
         <v>0</v>
@@ -7567,34 +7573,34 @@
         <v>0</v>
       </c>
       <c r="Y32" s="9" t="n">
-        <v>14.7</v>
+        <v>2.5</v>
       </c>
       <c r="Z32" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AA32" s="9" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="AB32" s="10" t="n">
-        <v>1308.9</v>
+        <v>1.2</v>
+      </c>
+      <c r="AB32" s="9" t="n">
+        <v>862.2</v>
       </c>
       <c r="AC32" s="10" t="n">
-        <v>19009.4</v>
+        <v>19462.1</v>
       </c>
       <c r="AD32" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE32" s="10" t="n">
-        <v>19009.4</v>
+        <v>19462.1</v>
       </c>
       <c r="AF32" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG32" s="10" t="n">
-        <v>16503.1</v>
+        <v>16896</v>
       </c>
       <c r="AH32" s="10" t="n">
-        <v>2503.8</v>
+        <v>2563.5</v>
       </c>
       <c r="AI32" s="9" t="n">
         <v>0</v>
@@ -7703,40 +7709,40 @@
         <v>0</v>
       </c>
       <c r="Y33" s="9" t="n">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="Z33" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AA33" s="9" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="AB33" s="9" t="n">
-        <v>226.7</v>
+        <v>108.7</v>
       </c>
       <c r="AC33" s="10" t="n">
-        <v>19700.6</v>
+        <v>19819.3</v>
       </c>
       <c r="AD33" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE33" s="10" t="n">
-        <v>19700.6</v>
+        <v>19819.3</v>
       </c>
       <c r="AF33" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG33" s="10" t="n">
-        <v>8843.700000000001</v>
+        <v>8896.9</v>
       </c>
       <c r="AH33" s="10" t="n">
-        <v>10844.3</v>
+        <v>10909.6</v>
       </c>
       <c r="AI33" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AJ33" s="9" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="AK33" s="9" t="n">
         <v>0</v>
@@ -7839,40 +7845,40 @@
         <v>0</v>
       </c>
       <c r="Y34" s="9" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="Z34" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AA34" s="9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AB34" s="9" t="n">
-        <v>38.5</v>
+        <v>13.6</v>
       </c>
       <c r="AC34" s="10" t="n">
-        <v>19879.7</v>
+        <v>19904.6</v>
       </c>
       <c r="AD34" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE34" s="10" t="n">
-        <v>19879.7</v>
+        <v>19904.6</v>
       </c>
       <c r="AF34" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG34" s="10" t="n">
-        <v>1834.9</v>
+        <v>1837.2</v>
       </c>
       <c r="AH34" s="10" t="n">
-        <v>17984</v>
+        <v>18006.5</v>
       </c>
       <c r="AI34" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AJ34" s="9" t="n">
-        <v>60.9</v>
+        <v>61</v>
       </c>
       <c r="AK34" s="9" t="n">
         <v>0</v>
@@ -7984,31 +7990,31 @@
         <v>0</v>
       </c>
       <c r="AB35" s="9" t="n">
-        <v>6.4</v>
+        <v>1.7</v>
       </c>
       <c r="AC35" s="10" t="n">
-        <v>19614.2</v>
+        <v>19618.9</v>
       </c>
       <c r="AD35" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE35" s="10" t="n">
-        <v>19614.2</v>
+        <v>19618.9</v>
       </c>
       <c r="AF35" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AG35" s="9" t="n">
-        <v>247.1</v>
+        <v>247.2</v>
       </c>
       <c r="AH35" s="10" t="n">
-        <v>19085.4</v>
+        <v>19090</v>
       </c>
       <c r="AI35" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AJ35" s="9" t="n">
-        <v>281.6</v>
+        <v>281.7</v>
       </c>
       <c r="AK35" s="9" t="n">
         <v>0</v>
@@ -8120,16 +8126,16 @@
         <v>0</v>
       </c>
       <c r="AB36" s="9" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="AC36" s="10" t="n">
-        <v>18842.7</v>
+        <v>18843.5</v>
       </c>
       <c r="AD36" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE36" s="10" t="n">
-        <v>18842.7</v>
+        <v>18843.5</v>
       </c>
       <c r="AF36" s="9" t="n">
         <v>0</v>
@@ -8138,13 +8144,13 @@
         <v>30</v>
       </c>
       <c r="AH36" s="10" t="n">
-        <v>17590.7</v>
+        <v>17591.4</v>
       </c>
       <c r="AI36" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AJ36" s="10" t="n">
-        <v>1222</v>
+        <v>1222.1</v>
       </c>
       <c r="AK36" s="9" t="n">
         <v>0</v>
@@ -8256,16 +8262,16 @@
         <v>0</v>
       </c>
       <c r="AB37" s="9" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="AC37" s="10" t="n">
-        <v>17916.2</v>
+        <v>17916.3</v>
       </c>
       <c r="AD37" s="9" t="n">
         <v>0</v>
       </c>
       <c r="AE37" s="10" t="n">
-        <v>17916.2</v>
+        <v>17916.3</v>
       </c>
       <c r="AF37" s="9" t="n">
         <v>0</v>
@@ -8274,7 +8280,7 @@
         <v>3.5</v>
       </c>
       <c r="AH37" s="10" t="n">
-        <v>13454.5</v>
+        <v>13454.6</v>
       </c>
       <c r="AI37" s="9" t="n">
         <v>0</v>
@@ -8413,10 +8419,10 @@
         <v>6440.7</v>
       </c>
       <c r="AI38" s="10" t="n">
-        <v>1947.5</v>
+        <v>1945.3</v>
       </c>
       <c r="AJ38" s="10" t="n">
-        <v>8031.6</v>
+        <v>8033.8</v>
       </c>
       <c r="AK38" s="9" t="n">
         <v>0</v>
@@ -8549,10 +8555,10 @@
         <v>1671.6</v>
       </c>
       <c r="AI39" s="10" t="n">
-        <v>2504.1</v>
+        <v>2501.4</v>
       </c>
       <c r="AJ39" s="10" t="n">
-        <v>9881.200000000001</v>
+        <v>9884</v>
       </c>
       <c r="AK39" s="9" t="n">
         <v>0</v>
@@ -8685,10 +8691,10 @@
         <v>304.7</v>
       </c>
       <c r="AI40" s="10" t="n">
-        <v>2832.5</v>
+        <v>2830.6</v>
       </c>
       <c r="AJ40" s="10" t="n">
-        <v>23569.4</v>
+        <v>23571.3</v>
       </c>
       <c r="AK40" s="9" t="n">
         <v>0</v>
@@ -8821,10 +8827,10 @@
         <v>9.5</v>
       </c>
       <c r="AI41" s="9" t="n">
-        <v>539.2</v>
+        <v>539.3</v>
       </c>
       <c r="AJ41" s="10" t="n">
-        <v>20780.8</v>
+        <v>20780.7</v>
       </c>
       <c r="AK41" s="9" t="n">
         <v>0</v>
@@ -8957,10 +8963,10 @@
         <v>0.3</v>
       </c>
       <c r="AI42" s="9" t="n">
-        <v>70.2</v>
+        <v>70.3</v>
       </c>
       <c r="AJ42" s="10" t="n">
-        <v>16171.2</v>
+        <v>16171.1</v>
       </c>
       <c r="AK42" s="9" t="n">
         <v>0</v>
@@ -9093,7 +9099,7 @@
         <v>0</v>
       </c>
       <c r="AI43" s="9" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="AJ43" s="10" t="n">
         <v>13788.8</v>
@@ -9517,16 +9523,16 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>80682</v>
+        <v>80835</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>14.21</v>
+        <v>14.23</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>16238</v>
+        <v>16275</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>16.24</v>
+        <v>16.28</v>
       </c>
       <c r="G6" s="9" t="n">
         <v>57</v>
@@ -9538,10 +9544,10 @@
         <v>125</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>0.056</v>
+        <v>0.055</v>
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
@@ -9561,31 +9567,31 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>68744</v>
+        <v>68595</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>12.11</v>
+        <v>12.08</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>13046</v>
+        <v>13017</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>13.05</v>
+        <v>13.02</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>46.2</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="I7" s="8" t="n">
         <v>199</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>0.244</v>
+        <v>0.238</v>
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
@@ -9605,13 +9611,13 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>81587</v>
+        <v>81613</v>
       </c>
       <c r="D8" s="9" t="n">
         <v>14.37</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>14698</v>
+        <v>14701</v>
       </c>
       <c r="F8" s="9" t="n">
         <v>14.7</v>
@@ -9620,16 +9626,16 @@
         <v>37.2</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I8" s="8" t="n">
         <v>277</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
@@ -9649,31 +9655,31 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>45715</v>
+        <v>45847</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>8.050000000000001</v>
+        <v>8.07</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>7907</v>
+        <v>7930</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>7.91</v>
+        <v>7.93</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>30.5</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="I9" s="8" t="n">
         <v>345</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>1.778</v>
+        <v>1.779</v>
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
@@ -9693,22 +9699,22 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>50683</v>
+        <v>50356</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>8.93</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>8529</v>
+        <v>8467</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>8.529999999999999</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>26.1</v>
+        <v>25.9</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="I10" s="8" t="n">
         <v>398</v>
@@ -9717,7 +9723,7 @@
         <v>451</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>2.279</v>
+        <v>2.295</v>
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
@@ -9737,16 +9743,16 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>90231</v>
+        <v>90396</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>15.89</v>
+        <v>15.92</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>14526</v>
+        <v>14553</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>14.53</v>
+        <v>14.55</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>19.3</v>
@@ -9781,13 +9787,13 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>7901</v>
+        <v>7894</v>
       </c>
       <c r="D12" s="9" t="n">
         <v>1.39</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="F12" s="9" t="n">
         <v>1.21</v>
@@ -9825,13 +9831,13 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>108256</v>
+        <v>108263</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>19.06</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>16180</v>
+        <v>16181</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>16.18</v>
@@ -9868,13 +9874,13 @@
         <v>567874</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>100.01</v>
+        <v>99.98999999999999</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>100000</v>
+        <v>99999</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>100.01</v>
+        <v>100</v>
       </c>
       <c r="G14" s="8" t="inlineStr"/>
       <c r="H14" s="8" t="inlineStr"/>
@@ -9920,7 +9926,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>60.81</v>
+        <v>60.68</v>
       </c>
     </row>
     <row r="3">
@@ -9930,7 +9936,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>67.56999999999999</v>
+        <v>67.42</v>
       </c>
     </row>
     <row r="4">
@@ -9940,7 +9946,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>14.74</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="5">
@@ -9950,7 +9956,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>16.75</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="6">
@@ -9960,7 +9966,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>47.67</v>
+        <v>47.58</v>
       </c>
     </row>
     <row r="7">
@@ -9970,7 +9976,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>39.78</v>
+        <v>39.7</v>
       </c>
     </row>
     <row r="8">
@@ -9980,7 +9986,7 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>8.1</v>
+        <v>8.09</v>
       </c>
     </row>
     <row r="9">
@@ -9990,7 +9996,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>12.87</v>
+        <v>12.85</v>
       </c>
     </row>
     <row r="10">
@@ -10000,7 +10006,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>12.39</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="11">
@@ -10010,7 +10016,7 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>22.72</v>
+        <v>22.59</v>
       </c>
     </row>
     <row r="12">
@@ -10020,7 +10026,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>9.09</v>
+        <v>9.039999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -10030,7 +10036,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>13.63</v>
+        <v>13.55</v>
       </c>
     </row>
     <row r="14">
@@ -10040,7 +10046,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>94.11</v>
+        <v>94.33</v>
       </c>
     </row>
     <row r="15">
@@ -10050,7 +10056,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>273.54</v>
+        <v>274.02</v>
       </c>
     </row>
     <row r="16">
@@ -10060,7 +10066,7 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>8.49</v>
+        <v>8.51</v>
       </c>
     </row>
     <row r="17">
@@ -10151,19 +10157,19 @@
         </is>
       </c>
       <c r="C2" s="9" t="n">
-        <v>8.1</v>
+        <v>8.09</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>153.3</v>
+        <v>152.8</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>83.3</v>
+        <v>82.8</v>
       </c>
       <c r="F2" s="9" t="n">
         <v>30</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>55.7</v>
+        <v>55.6</v>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
@@ -10183,19 +10189,19 @@
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>210.1</v>
+        <v>211.5</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>75.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>55.7</v>
+        <v>55.6</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>75.3</v>
+        <v>75.5</v>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
@@ -10215,19 +10221,19 @@
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>11.37</v>
+        <v>11.45</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>220.6</v>
+        <v>223.7</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>95.3</v>
+        <v>95.5</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>75.3</v>
+        <v>75.5</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>108</v>
+        <v>108.4</v>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
@@ -10247,19 +10253,19 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>4.45</v>
+        <v>4.44</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>205</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>128</v>
+        <v>128.4</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>108</v>
+        <v>108.4</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>120.3</v>
+        <v>120.6</v>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
@@ -10288,10 +10294,10 @@
         <v>175</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>120.3</v>
+        <v>120.6</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>136.1</v>
+        <v>136.4</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
@@ -10311,19 +10317,19 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>12.87</v>
+        <v>12.85</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>238.5</v>
+        <v>240</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>158.5</v>
+        <v>160</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>136.1</v>
+        <v>136.4</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>169.3</v>
+        <v>169.6</v>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
@@ -10343,19 +10349,19 @@
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>5.7</v>
+        <v>5.83</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>291.8</v>
+        <v>293.5</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>205</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>169.3</v>
+        <v>169.6</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>183.5</v>
+        <v>184</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
@@ -10375,19 +10381,19 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>21.21</v>
+        <v>21.14</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>315.2</v>
+        <v>315</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>205.2</v>
+        <v>205</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>183.5</v>
+        <v>184</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>233.6</v>
+        <v>234</v>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
@@ -10407,19 +10413,19 @@
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>3.1</v>
+        <v>3.11</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>334.6</v>
+        <v>334.7</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>253.6</v>
+        <v>254</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>233.6</v>
+        <v>234</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>240.7</v>
+        <v>241</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
@@ -10439,19 +10445,19 @@
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>7.35</v>
+        <v>7.46</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>312.6</v>
+        <v>313.9</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>260.7</v>
+        <v>261</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>240.7</v>
+        <v>241</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>257</v>
+        <v>257.6</v>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
@@ -10471,19 +10477,19 @@
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>7.61</v>
+        <v>7.58</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>366.3</v>
+        <v>366.4</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>277</v>
+        <v>277.6</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>257</v>
+        <v>257.6</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>273.5</v>
+        <v>274</v>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
@@ -10503,13 +10509,13 @@
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>5.04</v>
+        <v>4.91</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>260.7</v>
+        <v>261</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>222.6</v>
+        <v>223.9</v>
       </c>
       <c r="F13" s="8" t="inlineStr"/>
       <c r="G13" s="8" t="inlineStr"/>
@@ -10534,7 +10540,7 @@
         <v>1.27</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>75.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="E14" s="9" t="n">
         <v>45</v>
@@ -10587,10 +10593,10 @@
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>6.03</v>
+        <v>6.06</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>253.6</v>
+        <v>254</v>
       </c>
       <c r="E16" s="9" t="n">
         <v>60</v>
@@ -10615,10 +10621,10 @@
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>95.3</v>
+        <v>95.5</v>
       </c>
       <c r="E17" s="9" t="n">
         <v>55</v>
@@ -10643,10 +10649,10 @@
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>7.58</v>
+        <v>7.62</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>277</v>
+        <v>277.6</v>
       </c>
       <c r="E18" s="9" t="n">
         <v>175</v>
@@ -10674,7 +10680,7 @@
         <v>6.64</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>205.2</v>
+        <v>205</v>
       </c>
       <c r="E19" s="9" t="n">
         <v>90</v>

</xml_diff>

<commit_message>
PFDs (6 sheets), electrical package (load list, SLDs, calcs, cable schedule); fix preheat trim double-counting, E-114 balance, stream tags
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/00-basis/CFU-000-PR-HMB-001_Heat-Material-Balance.xlsx
+++ b/deliverables/00-basis/CFU-000-PR-HMB-001_Heat-Material-Balance.xlsx
@@ -1000,7 +1000,7 @@
       </c>
       <c r="Y5" s="4" t="inlineStr">
         <is>
-          <t>E-202</t>
+          <t>A-202</t>
         </is>
       </c>
       <c r="Z5" s="4" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>C-101/C-102A-C</t>
+          <t>C-101/C-102/C-103/C-104</t>
         </is>
       </c>
       <c r="V6" s="4" t="inlineStr">
@@ -10066,7 +10066,7 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>8.51</v>
+        <v>10.83</v>
       </c>
     </row>
     <row r="17">
@@ -10565,10 +10565,10 @@
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>8.16</v>
+        <v>3.72</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>205</v>
+        <v>128.4</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>55</v>
@@ -10649,13 +10649,13 @@
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>7.62</v>
+        <v>1.78</v>
       </c>
       <c r="D18" s="9" t="n">
         <v>277.6</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>175</v>
+        <v>255</v>
       </c>
       <c r="F18" s="8" t="inlineStr"/>
       <c r="G18" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
Mechanical package (calcs, datasheets, GAs); apply mechanical review to sizing
- C-201 bed-1 vapour load corrected (top ID 2.6 -> 4.4 m)
- H-201 efficiency 84 %, radiant fraction 0.70, heater box length fits 18.3 m tubes,
  heater design T per API 530 metal temperatures
- P-112 differential 17 bar, P-206 PD metering pump, air-cooler bays at 6 rows
- E-116/E-117 design T on steam supply, D-102 6 mm CA, X-104 area, C-101 swage
- D-103 relocated to keep 15 m from H-201

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/00-basis/CFU-000-PR-HMB-001_Heat-Material-Balance.xlsx
+++ b/deliverables/00-basis/CFU-000-PR-HMB-001_Heat-Material-Balance.xlsx
@@ -1732,7 +1732,7 @@
         <v>80835</v>
       </c>
       <c r="AI10" s="5" t="n">
-        <v>6443</v>
+        <v>6504</v>
       </c>
     </row>
     <row r="11">
@@ -2775,7 +2775,7 @@
       <c r="AG21" s="5" t="inlineStr"/>
       <c r="AH21" s="5" t="inlineStr"/>
       <c r="AI21" s="5" t="n">
-        <v>6443</v>
+        <v>6504</v>
       </c>
     </row>
     <row r="22">
@@ -2952,7 +2952,7 @@
       <c r="AG24" s="5" t="inlineStr"/>
       <c r="AH24" s="5" t="inlineStr"/>
       <c r="AI24" s="5" t="n">
-        <v>1804</v>
+        <v>1821</v>
       </c>
     </row>
     <row r="25">
@@ -9956,7 +9956,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>16.7</v>
+        <v>17.49</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
P&IDs (17 sheets), line list, instrument index, piping class summary; process fixes from P&ID review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/00-basis/CFU-000-PR-HMB-001_Heat-Material-Balance.xlsx
+++ b/deliverables/00-basis/CFU-000-PR-HMB-001_Heat-Material-Balance.xlsx
@@ -828,7 +828,7 @@
       </c>
       <c r="Z4" s="4" t="inlineStr">
         <is>
-          <t>Slop wax</t>
+          <t>Slop wax (hot, traced)</t>
         </is>
       </c>
       <c r="AA4" s="4" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="AA5" s="4" t="inlineStr">
         <is>
-          <t>E-201</t>
+          <t>E-105</t>
         </is>
       </c>
       <c r="AB5" s="4" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="Z6" s="4" t="inlineStr">
         <is>
-          <t>Slop / FCC</t>
+          <t>Delayed coker feed (hot)</t>
         </is>
       </c>
       <c r="AA6" s="4" t="inlineStr">
@@ -1487,7 +1487,7 @@
         <v>90</v>
       </c>
       <c r="Z8" s="5" t="n">
-        <v>90</v>
+        <v>378.4</v>
       </c>
       <c r="AA8" s="5" t="n">
         <v>175</v>
@@ -2596,7 +2596,7 @@
         <v>886.4</v>
       </c>
       <c r="Z19" s="5" t="n">
-        <v>934.2</v>
+        <v>713.6</v>
       </c>
       <c r="AA19" s="5" t="n">
         <v>904.8</v>
@@ -2685,7 +2685,7 @@
         <v>102</v>
       </c>
       <c r="Z20" s="5" t="n">
-        <v>8.4</v>
+        <v>11.1</v>
       </c>
       <c r="AA20" s="5" t="n">
         <v>119.7</v>
@@ -3022,7 +3022,7 @@
         <v>3619</v>
       </c>
       <c r="Z25" s="5" t="n">
-        <v>305</v>
+        <v>1922</v>
       </c>
       <c r="AA25" s="5" t="n">
         <v>9490</v>
@@ -9815,7 +9815,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>Slop / FCC</t>
+          <t>Delayed coker feed (hot)</t>
         </is>
       </c>
     </row>

</xml_diff>